<commit_message>
Add interactive HTML cleaning calendar alongside the Excel export.
Generate cleanings-{year}.html from bookings with per-day comments in localStorage, mobile-friendly scrolling layout, weekday palm toggles, and softer weekend shading.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/cleanings/templates/cleanings-map.xlsx
+++ b/cleanings/templates/cleanings-map.xlsx
@@ -920,7 +920,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="233">
+  <cellXfs count="236">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1532,6 +1532,11 @@
     <xf numFmtId="0" fontId="16" fillId="10" borderId="52" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>

</xml_diff>